<commit_message>
Add total column to team lead visits report
Co-authored-by: papie <papie@gonxt.tech>
</commit_message>
<xml_diff>
--- a/reports/team_lead_daily_visits.xlsx
+++ b/reports/team_lead_daily_visits.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -427,6 +427,7 @@
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -455,6 +456,11 @@
           <t>Gilda Katarina Mashele</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -474,6 +480,9 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,6 +502,9 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
+      <c r="F3" t="n">
+        <v>123</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -512,6 +524,9 @@
       <c r="E4" t="n">
         <v>0</v>
       </c>
+      <c r="F4" t="n">
+        <v>191</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -530,6 +545,9 @@
       </c>
       <c r="E5" t="n">
         <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>